<commit_message>
déplacer contenu dans cours précédent
</commit_message>
<xml_diff>
--- a/template/horaire.xlsx
+++ b/template/horaire.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/web3/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8831C609-8F45-6C4D-AD59-ADDDE634FAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F6FD58D-DB83-6B40-BF2A-4426B72ADE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="1580" windowWidth="25920" windowHeight="16440" xr2:uid="{4696F4E7-E751-AB46-8D30-A385E7EE1466}"/>
   </bookViews>
@@ -59,9 +59,6 @@
     <t>Retour sur formatif &lt;br/&gt; Période de questions</t>
   </si>
   <si>
-    <t>[Introduction à Next.js](lecons/next.js/introduction.md)</t>
-  </si>
-  <si>
     <t xml:space="preserve">[Introduction à TypeScript](lecons/typescript/introduction_typescript.md) &lt;br/&gt; [npm](lecons/typescript/npm.md) &lt;br/&gt;[Prettier](lecons/typescript/prettier.md)  </t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>Retour sur pratique d'examen final</t>
   </si>
   <si>
-    <t>[Routage dans Next.js](lecons/next.js/routage.md)</t>
-  </si>
-  <si>
     <t>[Modes de rendu](lecons/next.js/modes_rendu.md)</t>
   </si>
   <si>
@@ -192,6 +186,12 @@
   </si>
   <si>
     <t>Examen Next.js</t>
+  </si>
+  <si>
+    <t>[Introduction à Next.js](lecons/next.js/introduction.md) &lt;br/&gt;[Routage dans Next.js](lecons/next.js/routage.md)</t>
+  </si>
+  <si>
+    <t>**Exercice seulement**</t>
   </si>
 </sst>
 </file>
@@ -267,11 +267,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,10 +617,10 @@
         <v>46254.34375</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -630,10 +631,10 @@
         <v>46259.59375</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -644,10 +645,10 @@
         <v>46261.34375</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -658,10 +659,10 @@
         <v>46268.34375</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -672,10 +673,10 @@
         <v>46273.59375</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -686,10 +687,10 @@
         <v>46276.59375</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -700,10 +701,10 @@
         <v>46280.59375</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -714,10 +715,10 @@
         <v>46282.34375</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -728,10 +729,10 @@
         <v>46287.59375</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -742,10 +743,10 @@
         <v>46289.34375</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -778,10 +779,10 @@
         <v>46301.59375</v>
       </c>
       <c r="C14" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -791,11 +792,11 @@
       <c r="B15" s="2">
         <v>46303.34375</v>
       </c>
-      <c r="C15" t="s">
-        <v>19</v>
+      <c r="C15" s="4" t="s">
+        <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -817,10 +818,10 @@
         <v>46317.34375</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -831,10 +832,10 @@
         <v>46322.59375</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -845,10 +846,10 @@
         <v>46324.34375</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -859,10 +860,10 @@
         <v>46329.59375</v>
       </c>
       <c r="C20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -873,10 +874,10 @@
         <v>46331.34375</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -887,10 +888,10 @@
         <v>46338.34375</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -901,10 +902,10 @@
         <v>46343.59375</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -915,10 +916,10 @@
         <v>46345.34375</v>
       </c>
       <c r="C24" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -929,7 +930,7 @@
         <v>46350.59375</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -940,7 +941,7 @@
         <v>46352.34375</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -951,7 +952,7 @@
         <v>46357.59375</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -962,7 +963,7 @@
         <v>46359.34375</v>
       </c>
       <c r="C28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -973,7 +974,7 @@
         <v>46364.59375</v>
       </c>
       <c r="C29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -984,7 +985,7 @@
         <v>46366.34375</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -995,7 +996,7 @@
         <v>46371.59375</v>
       </c>
       <c r="C31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>